<commit_message>
Backup antes de ejecutar pipeline completo
Commit de seguridad antes de ejecutar Ejecutar_Pipeline_Completo.py
para validar la reorganización del proyecto Tesis_Ordenada.

🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/Resultados_Cleveland/Resumen_CO_Congruente_vs_Incongruente_Ballotage.xlsx
+++ b/Data/Resultados_Cleveland/Resumen_CO_Congruente_vs_Incongruente_Ballotage.xlsx
@@ -485,16 +485,16 @@
         <v>133</v>
       </c>
       <c r="D2" t="n">
-        <v>0.02255639097744361</v>
+        <v>0.003222341568206259</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.5789473684210527</v>
+        <v>-0.08270676691729323</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.6015037593984962</v>
+        <v>-0.08592910848549949</v>
       </c>
       <c r="G2" t="n">
-        <v>0.877352108907123</v>
+        <v>0.7307275902049302</v>
       </c>
       <c r="H2" t="inlineStr"/>
     </row>
@@ -513,16 +513,16 @@
         <v>597</v>
       </c>
       <c r="D3" t="n">
-        <v>0.5125628140703518</v>
+        <v>0.07322325915290738</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.169179229480737</v>
+        <v>-0.024168461354391</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.6817420435510888</v>
+        <v>-0.09739172050729838</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0094612312000834</v>
+        <v>0.008369660549967701</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -545,16 +545,16 @@
         <v>43</v>
       </c>
       <c r="D4" t="n">
-        <v>1.325581395348837</v>
+        <v>0.1893687707641195</v>
       </c>
       <c r="E4" t="n">
-        <v>0.4534883720930232</v>
+        <v>0.06478405315614616</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.8720930232558139</v>
+        <v>-0.1245847176079734</v>
       </c>
       <c r="G4" t="n">
-        <v>0.1631229948688568</v>
+        <v>0.1833803408752765</v>
       </c>
       <c r="H4" t="inlineStr"/>
     </row>
@@ -573,16 +573,16 @@
         <v>45</v>
       </c>
       <c r="D5" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.01904761904761905</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.3555555555555556</v>
+        <v>-0.05079365079365081</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.4888888888888889</v>
+        <v>-0.06984126984126986</v>
       </c>
       <c r="G5" t="n">
-        <v>0.3113185348688483</v>
+        <v>0.3124613036340934</v>
       </c>
       <c r="H5" t="inlineStr"/>
     </row>
@@ -601,16 +601,16 @@
         <v>116</v>
       </c>
       <c r="D6" t="n">
-        <v>0.3189655172413793</v>
+        <v>0.04556650246305418</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.418103448275862</v>
+        <v>-0.05972906403940887</v>
       </c>
       <c r="F6" t="n">
-        <v>-0.7370689655172413</v>
+        <v>-0.1052955665024631</v>
       </c>
       <c r="G6" t="n">
-        <v>0.4638870319227534</v>
+        <v>0.6663727518104029</v>
       </c>
       <c r="H6" t="inlineStr"/>
     </row>
@@ -629,16 +629,16 @@
         <v>93</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.08602150537634409</v>
+        <v>-0.01228878648233486</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.5698924731182796</v>
+        <v>-0.08141321044546852</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.4838709677419355</v>
+        <v>-0.06912442396313366</v>
       </c>
       <c r="G7" t="n">
-        <v>0.9943682088579749</v>
+        <v>0.9719816782101542</v>
       </c>
       <c r="H7" t="inlineStr"/>
     </row>

</xml_diff>